<commit_message>
feat: generate ppbr by hhincome
</commit_message>
<xml_diff>
--- a/output/five-decade-tables/crowding_percent_by_group - manual edit.xlsx
+++ b/output/five-decade-tables/crowding_percent_by_group - manual edit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\output\five-decade-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDB48D2-6D6A-4B63-AB97-044EFB6B3367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE1151E-A397-4652-A02A-C6E729AC199D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,7 +108,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="172" formatCode="0.0\%"/>
+    <numFmt numFmtId="164" formatCode="0.0\%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -184,23 +184,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -740,92 +741,92 @@
       <c r="A12" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="7">
-        <v>10.664587294436391</v>
-      </c>
-      <c r="C12" s="7">
-        <v>6.8380569619002536</v>
-      </c>
-      <c r="D12" s="7">
-        <v>8.247766684922107</v>
-      </c>
-      <c r="E12" s="7">
-        <v>10.219405368829859</v>
-      </c>
-      <c r="F12" s="7">
-        <v>5.6092620851298047</v>
-      </c>
-      <c r="G12" s="7">
-        <v>5.2576261875042629</v>
+      <c r="B12" s="10">
+        <v>19.685956645830579</v>
+      </c>
+      <c r="C12" s="10">
+        <v>11.56412506960371</v>
+      </c>
+      <c r="D12" s="10">
+        <v>12.819765157337461</v>
+      </c>
+      <c r="E12" s="10">
+        <v>14.40415035612742</v>
+      </c>
+      <c r="F12" s="10">
+        <v>8.6833102292296633</v>
+      </c>
+      <c r="G12" s="10">
+        <v>7.2792767408226782</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="7">
-        <v>6.9817828784314946</v>
-      </c>
-      <c r="C13" s="7">
-        <v>3.2603974114670371</v>
-      </c>
-      <c r="D13" s="7">
-        <v>3.153261927925294</v>
-      </c>
-      <c r="E13" s="7">
-        <v>3.6386637193751712</v>
-      </c>
-      <c r="F13" s="7">
-        <v>1.755590834728596</v>
-      </c>
-      <c r="G13" s="7">
-        <v>2.245082406545349</v>
+      <c r="B13" s="10">
+        <v>14.692699017289</v>
+      </c>
+      <c r="C13" s="10">
+        <v>7.9190910043676341</v>
+      </c>
+      <c r="D13" s="10">
+        <v>8.5078738514118069</v>
+      </c>
+      <c r="E13" s="10">
+        <v>11.09295128754513</v>
+      </c>
+      <c r="F13" s="10">
+        <v>6.1091567942114633</v>
+      </c>
+      <c r="G13" s="10">
+        <v>6.2513512914534362</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="7">
-        <v>3.8251625456788951</v>
-      </c>
-      <c r="C14" s="7">
-        <v>1.6717912529193339</v>
-      </c>
-      <c r="D14" s="7">
-        <v>1.5500244103533529</v>
-      </c>
-      <c r="E14" s="7">
-        <v>2.2356252633363498</v>
-      </c>
-      <c r="F14" s="7">
-        <v>1.0333734459554731</v>
-      </c>
-      <c r="G14" s="7">
-        <v>1.467309971027005</v>
+      <c r="B14" s="10">
+        <v>10.040358424937359</v>
+      </c>
+      <c r="C14" s="10">
+        <v>5.5939521110160442</v>
+      </c>
+      <c r="D14" s="10">
+        <v>6.1121167581407763</v>
+      </c>
+      <c r="E14" s="10">
+        <v>7.7121033346279004</v>
+      </c>
+      <c r="F14" s="10">
+        <v>4.1319371227363018</v>
+      </c>
+      <c r="G14" s="10">
+        <v>4.9567717273228968</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="9">
-        <v>2.3473971637452662</v>
-      </c>
-      <c r="C15" s="9">
-        <v>1.214413696993828</v>
-      </c>
-      <c r="D15" s="9">
-        <v>1.0617993764324101</v>
-      </c>
-      <c r="E15" s="9">
-        <v>1.6661003733583519</v>
-      </c>
-      <c r="F15" s="9">
-        <v>0.6446839140196241</v>
-      </c>
-      <c r="G15" s="9">
-        <v>1.072956562966523</v>
+      <c r="B15" s="10">
+        <v>7.7228499790501406</v>
+      </c>
+      <c r="C15" s="10">
+        <v>4.7560152912075564</v>
+      </c>
+      <c r="D15" s="10">
+        <v>4.7532877178001174</v>
+      </c>
+      <c r="E15" s="10">
+        <v>5.7242219431207042</v>
+      </c>
+      <c r="F15" s="10">
+        <v>2.8595143056352099</v>
+      </c>
+      <c r="G15" s="10">
+        <v>4.1556170055584412</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>